<commit_message>
Desactivacion del modo nitro por defecto en el modelo universal
</commit_message>
<xml_diff>
--- a/01.Documentation/Control de versiones de Sistema.xlsx
+++ b/01.Documentation/Control de versiones de Sistema.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Team Dropbox\JRODRIGUEZ\Repositorios\01.Rover\01.Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB364415-99B6-497E-A661-4474EDC44A10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{159FE98A-6F96-4990-B698-11DF2E9B2671}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{24CF4CE9-DAD2-45B7-A0D0-75488DFF3356}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{24CF4CE9-DAD2-45B7-A0D0-75488DFF3356}"/>
   </bookViews>
   <sheets>
     <sheet name="ROVER" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="81">
   <si>
     <t>Cambios</t>
   </si>
@@ -442,7 +442,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -560,17 +560,6 @@
       </left>
       <right/>
       <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
       <bottom/>
       <diagonal/>
     </border>
@@ -578,7 +567,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -640,9 +629,6 @@
     <xf numFmtId="49" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -652,6 +638,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -661,6 +668,15 @@
     <xf numFmtId="0" fontId="1" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -687,27 +703,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1023,263 +1018,278 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11BF0786-E6C7-4307-9339-45491EF3032D}">
-  <dimension ref="A1:S100"/>
+  <dimension ref="A1:T100"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" style="10" customWidth="1"/>
-    <col min="2" max="2" width="44.85546875" style="39" customWidth="1"/>
-    <col min="3" max="3" width="17.5703125" style="2" customWidth="1"/>
-    <col min="4" max="6" width="12.140625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="8" style="2" customWidth="1"/>
-    <col min="8" max="8" width="6.7109375" style="2" customWidth="1"/>
-    <col min="9" max="9" width="14.28515625" style="2" customWidth="1"/>
-    <col min="10" max="10" width="7.42578125" style="2" customWidth="1"/>
-    <col min="11" max="11" width="7.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="6.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="18.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="19" max="16384" width="11.42578125" style="2"/>
+    <col min="2" max="2" width="44.85546875" style="28" customWidth="1"/>
+    <col min="3" max="4" width="17.5703125" style="2" customWidth="1"/>
+    <col min="5" max="7" width="12.140625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="8" style="2" customWidth="1"/>
+    <col min="9" max="9" width="6.7109375" style="2" customWidth="1"/>
+    <col min="10" max="10" width="14.28515625" style="2" customWidth="1"/>
+    <col min="11" max="11" width="7.42578125" style="2" customWidth="1"/>
+    <col min="12" max="12" width="7.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="6.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8" style="2" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="20" max="16384" width="11.42578125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="36" t="s">
+    <row r="1" spans="1:20" ht="21" x14ac:dyDescent="0.25">
+      <c r="A1" s="45" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="30" t="s">
+      <c r="B1" s="45"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-    </row>
-    <row r="2" spans="1:19" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="31" t="s">
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+    </row>
+    <row r="2" spans="1:20" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="40" t="s">
         <v>38</v>
       </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31" t="s">
+      <c r="B2" s="40"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="40" t="s">
         <v>45</v>
       </c>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A3" s="24" t="s">
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A3" s="30" t="s">
         <v>39</v>
       </c>
-      <c r="B3" s="24"/>
-      <c r="C3" s="32" t="s">
+      <c r="B3" s="30"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-    </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A4" s="24" t="s">
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="41"/>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A4" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="32" t="s">
+      <c r="B4" s="30"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="41" t="s">
         <v>46</v>
       </c>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
-      <c r="F4" s="32"/>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A5" s="24" t="s">
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
+      <c r="G4" s="41"/>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A5" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="B5" s="24"/>
-      <c r="C5" s="32" t="s">
+      <c r="B5" s="30"/>
+      <c r="C5" s="23"/>
+      <c r="D5" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
-      <c r="F5" s="32"/>
-    </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A6" s="24" t="s">
+      <c r="E5" s="41"/>
+      <c r="F5" s="41"/>
+      <c r="G5" s="41"/>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A6" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="24"/>
-    </row>
-    <row r="7" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="8" spans="1:19" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="25" t="s">
+      <c r="B6" s="30"/>
+    </row>
+    <row r="7" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="1:20" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="31" t="s">
         <v>24</v>
       </c>
-      <c r="B8" s="40" t="s">
+      <c r="B8" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="C8" s="34" t="s">
+      <c r="C8" s="43" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="34"/>
-      <c r="E8" s="34"/>
-      <c r="F8" s="34"/>
-      <c r="G8" s="35" t="s">
+      <c r="D8" s="43"/>
+      <c r="E8" s="43"/>
+      <c r="F8" s="43"/>
+      <c r="G8" s="43"/>
+      <c r="H8" s="44" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="35"/>
-      <c r="I8" s="35"/>
-      <c r="J8" s="35"/>
-      <c r="K8" s="35"/>
-      <c r="L8" s="35"/>
-      <c r="M8" s="35"/>
-      <c r="N8" s="35"/>
-      <c r="O8" s="35"/>
-      <c r="P8" s="33" t="s">
+      <c r="I8" s="44"/>
+      <c r="J8" s="44"/>
+      <c r="K8" s="44"/>
+      <c r="L8" s="44"/>
+      <c r="M8" s="44"/>
+      <c r="N8" s="44"/>
+      <c r="O8" s="44"/>
+      <c r="P8" s="44"/>
+      <c r="Q8" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="Q8" s="33"/>
-      <c r="R8" s="33"/>
-      <c r="S8" s="28" t="s">
+      <c r="R8" s="42"/>
+      <c r="S8" s="42"/>
+      <c r="T8" s="37" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="26"/>
-      <c r="B9" s="41"/>
+    <row r="9" spans="1:20" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="32"/>
+      <c r="B9" s="35"/>
       <c r="C9" s="16" t="s">
         <v>23</v>
       </c>
       <c r="D9" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="16" t="s">
+      <c r="F9" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="F9" s="16" t="s">
+      <c r="G9" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="G9" s="17" t="s">
+      <c r="H9" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="H9" s="17" t="s">
+      <c r="I9" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="17" t="s">
+      <c r="J9" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="J9" s="17" t="s">
+      <c r="K9" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="K9" s="21" t="s">
+      <c r="L9" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="L9" s="17" t="s">
+      <c r="M9" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="M9" s="17" t="s">
+      <c r="N9" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="N9" s="17" t="s">
+      <c r="O9" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="O9" s="17" t="s">
+      <c r="P9" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="P9" s="18" t="s">
+      <c r="Q9" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="Q9" s="18" t="s">
+      <c r="R9" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="R9" s="18" t="s">
+      <c r="S9" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="S9" s="29"/>
-    </row>
-    <row r="10" spans="1:19" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="27"/>
-      <c r="B10" s="42"/>
+      <c r="T9" s="38"/>
+    </row>
+    <row r="10" spans="1:20" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="33"/>
+      <c r="B10" s="36"/>
       <c r="C10" s="4">
-        <f>MAX(C11:C37)</f>
+        <f>MAX(C11:C100)</f>
+        <v>400</v>
+      </c>
+      <c r="D10" s="4">
+        <f t="shared" ref="D10:H10" si="0">MAX(D11:D100)</f>
         <v>125</v>
-      </c>
-      <c r="D10" s="4">
-        <f t="shared" ref="D10:E10" si="0">MAX(D11:D37)</f>
-        <v>313</v>
       </c>
       <c r="E10" s="4">
         <f t="shared" si="0"/>
+        <v>313</v>
+      </c>
+      <c r="F10" s="4">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F10" s="4">
-        <f>MAX(F11:F37)</f>
+      <c r="G10" s="4">
+        <f t="shared" si="0"/>
         <v>205</v>
       </c>
-      <c r="G10" s="5">
-        <f>MAX(G11:G100)</f>
+      <c r="H10" s="5">
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="H10" s="5">
-        <f t="shared" ref="H10:O10" si="1">MAX(H11:H100)</f>
+      <c r="I10" s="5">
+        <f t="shared" ref="I10" si="1">MAX(I11:I100)</f>
         <v>6</v>
       </c>
-      <c r="I10" s="5">
-        <f t="shared" si="1"/>
+      <c r="J10" s="5">
+        <f t="shared" ref="J10" si="2">MAX(J11:J100)</f>
         <v>3</v>
       </c>
-      <c r="J10" s="5">
-        <f t="shared" si="1"/>
+      <c r="K10" s="5">
+        <f t="shared" ref="K10:L10" si="3">MAX(K11:K100)</f>
         <v>1</v>
       </c>
-      <c r="K10" s="22">
-        <f t="shared" si="1"/>
+      <c r="L10" s="5">
+        <f t="shared" si="3"/>
         <v>2</v>
       </c>
-      <c r="L10" s="5">
-        <f t="shared" si="1"/>
+      <c r="M10" s="5">
+        <f t="shared" ref="M10" si="4">MAX(M11:M100)</f>
         <v>1</v>
       </c>
-      <c r="M10" s="5">
-        <f t="shared" si="1"/>
+      <c r="N10" s="5">
+        <f t="shared" ref="N10" si="5">MAX(N11:N100)</f>
         <v>3</v>
       </c>
-      <c r="N10" s="5">
-        <f t="shared" si="1"/>
+      <c r="O10" s="5">
+        <f t="shared" ref="O10" si="6">MAX(O11:O100)</f>
         <v>7</v>
       </c>
-      <c r="O10" s="5">
-        <f t="shared" si="1"/>
+      <c r="P10" s="5">
+        <f t="shared" ref="P10:Q10" si="7">MAX(P11:P100)</f>
         <v>1</v>
       </c>
-      <c r="P10" s="6">
-        <f>MAX(P11:P100)</f>
+      <c r="Q10" s="6">
+        <f>MAX(Q11:Q100)</f>
         <v>5</v>
       </c>
-      <c r="Q10" s="6">
-        <f t="shared" ref="Q10:R10" si="2">MAX(Q11:Q100)</f>
+      <c r="R10" s="6">
+        <f t="shared" ref="R10:S10" si="8">MAX(R11:R100)</f>
         <v>11</v>
       </c>
-      <c r="R10" s="6">
-        <f t="shared" si="2"/>
+      <c r="S10" s="6">
+        <f t="shared" si="8"/>
         <v>14</v>
       </c>
-      <c r="S10" s="15"/>
-    </row>
-    <row r="11" spans="1:19" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="T10" s="15"/>
+    </row>
+    <row r="11" spans="1:20" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="37" t="s">
+      <c r="B11" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="1"/>
+      <c r="C11" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="D11" s="1"/>
-      <c r="E11" s="1" t="s">
+      <c r="E11" s="1"/>
+      <c r="F11" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F11" s="1"/>
       <c r="G11" s="1"/>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
@@ -1292,21 +1302,24 @@
       <c r="P11" s="1"/>
       <c r="Q11" s="1"/>
       <c r="R11" s="1"/>
-      <c r="S11" s="7"/>
-    </row>
-    <row r="12" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="S11" s="1"/>
+      <c r="T11" s="7"/>
+    </row>
+    <row r="12" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="37" t="s">
+      <c r="B12" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="1"/>
+      <c r="C12" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="D12" s="1"/>
-      <c r="E12" s="1" t="s">
+      <c r="E12" s="1"/>
+      <c r="F12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F12" s="1"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
@@ -1319,21 +1332,24 @@
       <c r="P12" s="1"/>
       <c r="Q12" s="1"/>
       <c r="R12" s="1"/>
-      <c r="S12" s="7"/>
-    </row>
-    <row r="13" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="S12" s="1"/>
+      <c r="T12" s="7"/>
+    </row>
+    <row r="13" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="37" t="s">
+      <c r="B13" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="1"/>
+      <c r="C13" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="D13" s="1"/>
-      <c r="E13" s="1" t="s">
+      <c r="E13" s="1"/>
+      <c r="F13" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F13" s="1"/>
       <c r="G13" s="1"/>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
@@ -1346,77 +1362,81 @@
       <c r="P13" s="1"/>
       <c r="Q13" s="1"/>
       <c r="R13" s="1"/>
-      <c r="S13" s="7"/>
-    </row>
-    <row r="14" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="S13" s="1"/>
+      <c r="T13" s="7"/>
+    </row>
+    <row r="14" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="B14" s="37" t="s">
+      <c r="B14" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="13">
-        <v>121</v>
+      <c r="C14" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="D14" s="13">
         <v>121</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="E14" s="13">
+        <v>121</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F14" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G14" s="1">
-        <v>5</v>
+      <c r="G14" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="H14" s="1">
         <v>5</v>
       </c>
       <c r="I14" s="1">
+        <v>5</v>
+      </c>
+      <c r="J14" s="1">
         <v>2</v>
       </c>
-      <c r="J14" s="1">
+      <c r="K14" s="1">
         <v>1</v>
       </c>
-      <c r="K14" s="1"/>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
       <c r="N14" s="1"/>
       <c r="O14" s="1"/>
-      <c r="P14" s="1">
+      <c r="P14" s="1"/>
+      <c r="Q14" s="1">
         <v>5</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="R14" s="1">
         <v>9</v>
       </c>
-      <c r="R14" s="1">
+      <c r="S14" s="1">
         <v>10</v>
       </c>
-      <c r="S14" s="7"/>
-    </row>
-    <row r="15" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="T14" s="7"/>
+    </row>
+    <row r="15" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="B15" s="37" t="s">
+      <c r="B15" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="1" t="s">
         <v>13</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="E15" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F15" s="13">
+      <c r="G15" s="13">
         <v>201</v>
       </c>
-      <c r="G15" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="H15" s="1" t="s">
         <v>13</v>
       </c>
@@ -1426,41 +1446,44 @@
       <c r="J15" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="K15" s="1"/>
+      <c r="K15" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
       <c r="N15" s="1"/>
       <c r="O15" s="1"/>
-      <c r="P15" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="P15" s="1"/>
       <c r="Q15" s="1" t="s">
         <v>13</v>
       </c>
       <c r="R15" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="S15" s="7"/>
-    </row>
-    <row r="16" spans="1:19" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="S15" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="T15" s="7"/>
+    </row>
+    <row r="16" spans="1:20" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A16" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="38" t="s">
+      <c r="B16" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="1" t="s">
         <v>13</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="E16" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F16" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="G16" s="1" t="s">
         <v>13</v>
       </c>
@@ -1473,41 +1496,44 @@
       <c r="J16" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="K16" s="1"/>
+      <c r="K16" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="L16" s="1"/>
       <c r="M16" s="1"/>
       <c r="N16" s="1"/>
       <c r="O16" s="1"/>
-      <c r="P16" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="P16" s="1"/>
       <c r="Q16" s="1" t="s">
         <v>13</v>
       </c>
       <c r="R16" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="S16" s="7"/>
-    </row>
-    <row r="17" spans="1:19" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="S16" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="T16" s="7"/>
+    </row>
+    <row r="17" spans="1:20" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A17" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="B17" s="38" t="s">
+      <c r="B17" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="1" t="s">
         <v>13</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="E17" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F17" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F17" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="G17" s="1" t="s">
         <v>13</v>
       </c>
@@ -1520,41 +1546,44 @@
       <c r="J17" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="K17" s="1"/>
+      <c r="K17" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="L17" s="1"/>
       <c r="M17" s="1"/>
       <c r="N17" s="1"/>
       <c r="O17" s="1"/>
-      <c r="P17" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="P17" s="1"/>
       <c r="Q17" s="1" t="s">
         <v>13</v>
       </c>
       <c r="R17" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="S17" s="7"/>
-    </row>
-    <row r="18" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="S17" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="T17" s="7"/>
+    </row>
+    <row r="18" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="37" t="s">
+      <c r="B18" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="C18" s="13">
-        <v>122</v>
+      <c r="C18" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="D18" s="13">
         <v>122</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="E18" s="13">
+        <v>122</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F18" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="G18" s="1" t="s">
         <v>13</v>
       </c>
@@ -1567,27 +1596,30 @@
       <c r="J18" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="K18" s="1"/>
+      <c r="K18" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="L18" s="1"/>
       <c r="M18" s="1"/>
       <c r="N18" s="1"/>
       <c r="O18" s="1"/>
-      <c r="P18" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="P18" s="1"/>
       <c r="Q18" s="1" t="s">
         <v>13</v>
       </c>
       <c r="R18" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="S18" s="7"/>
-    </row>
-    <row r="19" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="S18" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="T18" s="7"/>
+    </row>
+    <row r="19" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="B19" s="37" t="s">
+      <c r="B19" s="26" t="s">
         <v>19</v>
       </c>
       <c r="C19" s="1" t="s">
@@ -1597,14 +1629,14 @@
         <v>13</v>
       </c>
       <c r="E19" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F19" s="13">
+      <c r="G19" s="13">
         <v>202</v>
       </c>
-      <c r="G19" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="H19" s="1" t="s">
         <v>13</v>
       </c>
@@ -1614,41 +1646,44 @@
       <c r="J19" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="K19" s="1"/>
+      <c r="K19" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="L19" s="1"/>
       <c r="M19" s="1"/>
       <c r="N19" s="1"/>
       <c r="O19" s="1"/>
-      <c r="P19" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="P19" s="1"/>
       <c r="Q19" s="1" t="s">
         <v>13</v>
       </c>
       <c r="R19" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="S19" s="7"/>
-    </row>
-    <row r="20" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="S19" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="T19" s="7"/>
+    </row>
+    <row r="20" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="B20" s="37" t="s">
+      <c r="B20" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="C20" s="13">
-        <v>123</v>
+      <c r="C20" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="D20" s="13">
         <v>123</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="E20" s="13">
+        <v>123</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F20" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="G20" s="1" t="s">
         <v>13</v>
       </c>
@@ -1661,27 +1696,30 @@
       <c r="J20" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="K20" s="1"/>
+      <c r="K20" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="L20" s="1"/>
       <c r="M20" s="1"/>
       <c r="N20" s="1"/>
       <c r="O20" s="1"/>
-      <c r="P20" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="P20" s="1"/>
       <c r="Q20" s="1" t="s">
         <v>13</v>
       </c>
       <c r="R20" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="S20" s="7"/>
-    </row>
-    <row r="21" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="S20" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="T20" s="7"/>
+    </row>
+    <row r="21" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="B21" s="37" t="s">
+      <c r="B21" s="26" t="s">
         <v>43</v>
       </c>
       <c r="C21" s="1" t="s">
@@ -1691,14 +1729,14 @@
         <v>13</v>
       </c>
       <c r="E21" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F21" s="13">
+      <c r="G21" s="13">
         <v>203</v>
       </c>
-      <c r="G21" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="H21" s="1" t="s">
         <v>13</v>
       </c>
@@ -1708,42 +1746,45 @@
       <c r="J21" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="K21" s="1"/>
+      <c r="K21" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="L21" s="1"/>
       <c r="M21" s="1"/>
       <c r="N21" s="1"/>
       <c r="O21" s="1"/>
-      <c r="P21" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="P21" s="1"/>
       <c r="Q21" s="1" t="s">
         <v>13</v>
       </c>
       <c r="R21" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="S21" s="7"/>
-    </row>
-    <row r="22" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+      <c r="S21" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="T21" s="7"/>
+    </row>
+    <row r="22" spans="1:20" ht="60" x14ac:dyDescent="0.25">
       <c r="A22" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="B22" s="37" t="s">
+      <c r="B22" s="26" t="s">
         <v>49</v>
       </c>
-      <c r="C22" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D22" s="14">
+      <c r="C22" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E22" s="14">
         <v>310</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="F22" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="F22" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G22" s="1" t="s">
+      <c r="G22" s="3" t="s">
         <v>13</v>
       </c>
       <c r="H22" s="1" t="s">
@@ -1755,74 +1796,80 @@
       <c r="J22" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="K22" s="1"/>
+      <c r="K22" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="L22" s="1"/>
       <c r="M22" s="1"/>
       <c r="N22" s="1"/>
       <c r="O22" s="1"/>
-      <c r="P22" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="P22" s="1"/>
       <c r="Q22" s="1" t="s">
         <v>13</v>
       </c>
       <c r="R22" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="S22" s="7"/>
-    </row>
-    <row r="23" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="S22" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="T22" s="7"/>
+    </row>
+    <row r="23" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="B23" s="37" t="s">
+      <c r="B23" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="C23" s="13">
+      <c r="C23" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" s="13">
         <v>123</v>
       </c>
-      <c r="D23" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="E23" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F23" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F23" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G23" s="13">
+      <c r="G23" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H23" s="13">
         <v>6</v>
       </c>
-      <c r="H23" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="I23" s="1" t="s">
         <v>13</v>
       </c>
       <c r="J23" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="K23" s="1"/>
+      <c r="K23" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="L23" s="1"/>
       <c r="M23" s="1"/>
       <c r="N23" s="1"/>
       <c r="O23" s="1"/>
-      <c r="P23" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="P23" s="1"/>
       <c r="Q23" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="R23" s="13">
+      <c r="R23" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="S23" s="13">
         <v>11</v>
       </c>
-      <c r="S23" s="7"/>
-    </row>
-    <row r="24" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="T23" s="7"/>
+    </row>
+    <row r="24" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="37" t="s">
+      <c r="B24" s="26" t="s">
         <v>50</v>
       </c>
       <c r="C24" s="1" t="s">
@@ -1832,105 +1879,111 @@
         <v>13</v>
       </c>
       <c r="E24" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F24" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F24" s="13">
+      <c r="G24" s="13">
         <v>203</v>
       </c>
-      <c r="G24" s="13">
+      <c r="H24" s="13">
         <v>6</v>
       </c>
-      <c r="H24" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="I24" s="1" t="s">
         <v>13</v>
       </c>
       <c r="J24" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="K24" s="1"/>
+      <c r="K24" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="L24" s="1"/>
       <c r="M24" s="1"/>
       <c r="N24" s="1"/>
       <c r="O24" s="1"/>
-      <c r="P24" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="P24" s="1"/>
       <c r="Q24" s="1" t="s">
         <v>13</v>
       </c>
       <c r="R24" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="S24" s="7"/>
-    </row>
-    <row r="25" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="S24" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="T24" s="7"/>
+    </row>
+    <row r="25" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="B25" s="37" t="s">
+      <c r="B25" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="C25" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D25" s="14">
+      <c r="C25" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E25" s="14">
         <v>310</v>
       </c>
-      <c r="E25" s="3" t="s">
+      <c r="F25" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="F25" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G25" s="13">
+      <c r="G25" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H25" s="13">
         <v>6</v>
       </c>
-      <c r="H25" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="I25" s="1" t="s">
         <v>13</v>
       </c>
       <c r="J25" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="K25" s="1"/>
+      <c r="K25" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="L25" s="1"/>
       <c r="M25" s="1"/>
       <c r="N25" s="1"/>
       <c r="O25" s="1"/>
-      <c r="P25" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="P25" s="1"/>
       <c r="Q25" s="1" t="s">
         <v>13</v>
       </c>
       <c r="R25" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="S25" s="7"/>
-    </row>
-    <row r="26" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="S25" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="T25" s="7"/>
+    </row>
+    <row r="26" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="B26" s="37" t="s">
+      <c r="B26" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="C26" s="13">
+      <c r="C26" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D26" s="13">
         <v>124</v>
       </c>
-      <c r="D26" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="E26" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F26" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F26" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="G26" s="1" t="s">
         <v>13</v>
       </c>
@@ -1943,27 +1996,30 @@
       <c r="J26" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="K26" s="1"/>
+      <c r="K26" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="L26" s="1"/>
       <c r="M26" s="1"/>
       <c r="N26" s="1"/>
       <c r="O26" s="1"/>
-      <c r="P26" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="P26" s="1"/>
       <c r="Q26" s="1" t="s">
         <v>13</v>
       </c>
       <c r="R26" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="S26" s="7"/>
-    </row>
-    <row r="27" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="S26" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="T26" s="7"/>
+    </row>
+    <row r="27" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="B27" s="37" t="s">
+      <c r="B27" s="26" t="s">
         <v>54</v>
       </c>
       <c r="C27" s="1" t="s">
@@ -1973,14 +2029,14 @@
         <v>13</v>
       </c>
       <c r="E27" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F27" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F27" s="13">
+      <c r="G27" s="13">
         <v>204</v>
       </c>
-      <c r="G27" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="H27" s="1" t="s">
         <v>13</v>
       </c>
@@ -1990,42 +2046,45 @@
       <c r="J27" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="K27" s="1"/>
+      <c r="K27" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
       <c r="N27" s="1"/>
       <c r="O27" s="1"/>
-      <c r="P27" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="P27" s="1"/>
       <c r="Q27" s="1" t="s">
         <v>13</v>
       </c>
       <c r="R27" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="S27" s="7"/>
-    </row>
-    <row r="28" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="S27" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="T27" s="7"/>
+    </row>
+    <row r="28" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="B28" s="37" t="s">
+      <c r="B28" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="C28" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D28" s="14">
+      <c r="C28" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E28" s="14">
         <v>311</v>
       </c>
-      <c r="E28" s="3" t="s">
+      <c r="F28" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="F28" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G28" s="1" t="s">
+      <c r="G28" s="3" t="s">
         <v>13</v>
       </c>
       <c r="H28" s="1" t="s">
@@ -2037,42 +2096,45 @@
       <c r="J28" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="K28" s="1"/>
+      <c r="K28" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
       <c r="N28" s="1"/>
       <c r="O28" s="1"/>
-      <c r="P28" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="P28" s="1"/>
       <c r="Q28" s="1" t="s">
         <v>13</v>
       </c>
       <c r="R28" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="S28" s="7"/>
-    </row>
-    <row r="29" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="S28" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="T28" s="7"/>
+    </row>
+    <row r="29" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="B29" s="37" t="s">
+      <c r="B29" s="26" t="s">
         <v>58</v>
       </c>
-      <c r="C29" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D29" s="14">
+      <c r="C29" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E29" s="14">
         <v>312</v>
       </c>
-      <c r="E29" s="3" t="s">
+      <c r="F29" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="F29" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G29" s="1" t="s">
+      <c r="G29" s="3" t="s">
         <v>13</v>
       </c>
       <c r="H29" s="1" t="s">
@@ -2084,55 +2146,58 @@
       <c r="J29" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="K29" s="1"/>
+      <c r="K29" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
       <c r="N29" s="1"/>
       <c r="O29" s="1"/>
-      <c r="P29" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="P29" s="1"/>
       <c r="Q29" s="1" t="s">
         <v>13</v>
       </c>
       <c r="R29" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="S29" s="7"/>
-    </row>
-    <row r="30" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="S29" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="T29" s="7"/>
+    </row>
+    <row r="30" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="B30" s="37" t="s">
+      <c r="B30" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="C30" s="14">
+      <c r="C30" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D30" s="14">
         <v>125</v>
       </c>
-      <c r="D30" s="3" t="s">
-        <v>13</v>
-      </c>
       <c r="E30" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F30" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="F30" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G30" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="H30" s="14">
+      <c r="G30" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H30" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I30" s="14">
         <v>6</v>
       </c>
-      <c r="I30" s="14">
+      <c r="J30" s="14">
         <v>3</v>
       </c>
-      <c r="J30" s="14">
+      <c r="K30" s="14">
         <v>1</v>
-      </c>
-      <c r="K30" s="3" t="s">
-        <v>22</v>
       </c>
       <c r="L30" s="3" t="s">
         <v>22</v>
@@ -2146,50 +2211,53 @@
       <c r="O30" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="P30" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q30" s="3">
+      <c r="P30" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q30" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="R30" s="3">
         <v>10</v>
       </c>
-      <c r="R30" s="3">
+      <c r="S30" s="3">
         <v>12</v>
       </c>
-      <c r="S30" s="7"/>
-    </row>
-    <row r="31" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="T30" s="7"/>
+    </row>
+    <row r="31" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="B31" s="37" t="s">
+      <c r="B31" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="C31" s="3" t="s">
+      <c r="C31" s="1" t="s">
         <v>13</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>13</v>
       </c>
       <c r="E31" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F31" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="F31" s="14">
+      <c r="G31" s="14">
         <v>205</v>
       </c>
-      <c r="G31" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="H31" s="14">
+      <c r="H31" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I31" s="14">
         <v>6</v>
       </c>
-      <c r="I31" s="14">
+      <c r="J31" s="14">
         <v>3</v>
       </c>
-      <c r="J31" s="14">
+      <c r="K31" s="14">
         <v>1</v>
-      </c>
-      <c r="K31" s="3" t="s">
-        <v>22</v>
       </c>
       <c r="L31" s="3" t="s">
         <v>22</v>
@@ -2203,50 +2271,53 @@
       <c r="O31" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="P31" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q31" s="3">
+      <c r="P31" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q31" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="R31" s="3">
         <v>10</v>
       </c>
-      <c r="R31" s="3">
+      <c r="S31" s="3">
         <v>12</v>
       </c>
-      <c r="S31" s="7"/>
-    </row>
-    <row r="32" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="T31" s="7"/>
+    </row>
+    <row r="32" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="B32" s="37" t="s">
+      <c r="B32" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="C32" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D32" s="14">
+      <c r="C32" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E32" s="14">
         <v>313</v>
       </c>
-      <c r="E32" s="3" t="s">
+      <c r="F32" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="F32" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G32" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="H32" s="14">
+      <c r="G32" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I32" s="14">
         <v>6</v>
       </c>
-      <c r="I32" s="14">
+      <c r="J32" s="14">
         <v>3</v>
       </c>
-      <c r="J32" s="14">
+      <c r="K32" s="14">
         <v>1</v>
-      </c>
-      <c r="K32" s="3" t="s">
-        <v>22</v>
       </c>
       <c r="L32" s="3" t="s">
         <v>22</v>
@@ -2260,82 +2331,88 @@
       <c r="O32" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="P32" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q32" s="3">
+      <c r="P32" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q32" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="R32" s="3">
         <v>10</v>
       </c>
-      <c r="R32" s="3">
+      <c r="S32" s="3">
         <v>12</v>
       </c>
-      <c r="S32" s="7"/>
-    </row>
-    <row r="33" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="T32" s="7"/>
+    </row>
+    <row r="33" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="B33" s="37" t="s">
+      <c r="B33" s="26" t="s">
         <v>61</v>
       </c>
-      <c r="C33" s="14">
+      <c r="C33" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D33" s="14">
         <v>125</v>
       </c>
-      <c r="D33" s="3" t="s">
-        <v>13</v>
-      </c>
       <c r="E33" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F33" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="F33" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G33" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="H33" s="14">
+      <c r="G33" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H33" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I33" s="14">
         <v>6</v>
       </c>
-      <c r="I33" s="14">
+      <c r="J33" s="14">
         <v>3</v>
       </c>
-      <c r="J33" s="14">
+      <c r="K33" s="14">
         <v>1</v>
       </c>
-      <c r="K33" s="14">
+      <c r="L33" s="14">
         <v>2</v>
       </c>
-      <c r="L33" s="14">
+      <c r="M33" s="14">
         <v>1</v>
       </c>
-      <c r="M33" s="14">
+      <c r="N33" s="14">
         <v>3</v>
       </c>
-      <c r="N33" s="14">
+      <c r="O33" s="14">
         <v>7</v>
       </c>
-      <c r="O33" s="14">
+      <c r="P33" s="14">
         <v>1</v>
       </c>
-      <c r="P33" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q33" s="3">
+      <c r="Q33" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="R33" s="3">
         <v>10</v>
       </c>
-      <c r="R33" s="3">
+      <c r="S33" s="3">
         <v>12</v>
       </c>
-      <c r="S33" s="7"/>
-    </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T33" s="7"/>
+    </row>
+    <row r="34" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="B34" s="37" t="s">
+      <c r="B34" s="26" t="s">
         <v>75</v>
       </c>
-      <c r="C34" s="3" t="s">
+      <c r="C34" s="1" t="s">
         <v>13</v>
       </c>
       <c r="D34" s="3" t="s">
@@ -2347,12 +2424,12 @@
       <c r="F34" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G34" s="23">
+      <c r="G34" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H34" s="22">
         <v>8</v>
       </c>
-      <c r="H34" s="3" t="s">
-        <v>13</v>
-      </c>
       <c r="I34" s="3" t="s">
         <v>13</v>
       </c>
@@ -2380,19 +2457,22 @@
       <c r="Q34" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="R34" s="3">
-        <v>13</v>
-      </c>
-      <c r="S34" s="7"/>
-    </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="R34" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="S34" s="3">
+        <v>13</v>
+      </c>
+      <c r="T34" s="7"/>
+    </row>
+    <row r="35" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="B35" s="37" t="s">
+      <c r="B35" s="26" t="s">
         <v>75</v>
       </c>
-      <c r="C35" s="3" t="s">
+      <c r="C35" s="1" t="s">
         <v>13</v>
       </c>
       <c r="D35" s="3" t="s">
@@ -2404,12 +2484,12 @@
       <c r="F35" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G35" s="23">
+      <c r="G35" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H35" s="22">
         <v>8</v>
       </c>
-      <c r="H35" s="3" t="s">
-        <v>13</v>
-      </c>
       <c r="I35" s="3" t="s">
         <v>13</v>
       </c>
@@ -2437,19 +2517,22 @@
       <c r="Q35" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="R35" s="3">
-        <v>13</v>
-      </c>
-      <c r="S35" s="7"/>
-    </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="R35" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="S35" s="3">
+        <v>13</v>
+      </c>
+      <c r="T35" s="7"/>
+    </row>
+    <row r="36" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="B36" s="37" t="s">
+      <c r="B36" s="26" t="s">
         <v>75</v>
       </c>
-      <c r="C36" s="3" t="s">
+      <c r="C36" s="1" t="s">
         <v>13</v>
       </c>
       <c r="D36" s="3" t="s">
@@ -2461,12 +2544,12 @@
       <c r="F36" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G36" s="23">
+      <c r="G36" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H36" s="22">
         <v>8</v>
       </c>
-      <c r="H36" s="3" t="s">
-        <v>13</v>
-      </c>
       <c r="I36" s="3" t="s">
         <v>13</v>
       </c>
@@ -2494,19 +2577,22 @@
       <c r="Q36" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="R36" s="3">
-        <v>13</v>
-      </c>
-      <c r="S36" s="7"/>
-    </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="R36" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="S36" s="3">
+        <v>13</v>
+      </c>
+      <c r="T36" s="7"/>
+    </row>
+    <row r="37" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A37" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="B37" s="37" t="s">
+      <c r="B37" s="26" t="s">
         <v>75</v>
       </c>
-      <c r="C37" s="3" t="s">
+      <c r="C37" s="1" t="s">
         <v>13</v>
       </c>
       <c r="D37" s="3" t="s">
@@ -2518,12 +2604,12 @@
       <c r="F37" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G37" s="23">
+      <c r="G37" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H37" s="22">
         <v>8</v>
       </c>
-      <c r="H37" s="3" t="s">
-        <v>13</v>
-      </c>
       <c r="I37" s="3" t="s">
         <v>13</v>
       </c>
@@ -2551,19 +2637,22 @@
       <c r="Q37" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="R37" s="3">
-        <v>13</v>
-      </c>
-      <c r="S37" s="7"/>
-    </row>
-    <row r="38" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="R37" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="S37" s="3">
+        <v>13</v>
+      </c>
+      <c r="T37" s="7"/>
+    </row>
+    <row r="38" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="B38" s="37" t="s">
+      <c r="B38" s="26" t="s">
         <v>80</v>
       </c>
-      <c r="C38" s="3" t="s">
+      <c r="C38" s="1" t="s">
         <v>13</v>
       </c>
       <c r="D38" s="3" t="s">
@@ -2605,22 +2694,25 @@
       <c r="P38" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="Q38" s="23">
+      <c r="Q38" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="R38" s="22">
         <v>11</v>
       </c>
-      <c r="R38" s="23">
+      <c r="S38" s="22">
         <v>14</v>
       </c>
-      <c r="S38" s="7"/>
-    </row>
-    <row r="39" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="T38" s="7"/>
+    </row>
+    <row r="39" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="B39" s="37" t="s">
+      <c r="B39" s="26" t="s">
         <v>80</v>
       </c>
-      <c r="C39" s="3" t="s">
+      <c r="C39" s="1" t="s">
         <v>13</v>
       </c>
       <c r="D39" s="3" t="s">
@@ -2662,22 +2754,25 @@
       <c r="P39" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="Q39" s="23">
+      <c r="Q39" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="R39" s="22">
         <v>11</v>
       </c>
-      <c r="R39" s="23">
+      <c r="S39" s="22">
         <v>14</v>
       </c>
-      <c r="S39" s="7"/>
-    </row>
-    <row r="40" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="T39" s="7"/>
+    </row>
+    <row r="40" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="B40" s="37" t="s">
+      <c r="B40" s="26" t="s">
         <v>80</v>
       </c>
-      <c r="C40" s="3" t="s">
+      <c r="C40" s="1" t="s">
         <v>13</v>
       </c>
       <c r="D40" s="3" t="s">
@@ -2719,23 +2814,26 @@
       <c r="P40" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="Q40" s="23">
+      <c r="Q40" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="R40" s="22">
         <v>11</v>
       </c>
-      <c r="R40" s="23">
+      <c r="S40" s="22">
         <v>14</v>
       </c>
-      <c r="S40" s="7"/>
-    </row>
-    <row r="41" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="T40" s="7"/>
+    </row>
+    <row r="41" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="19" t="s">
         <v>79</v>
       </c>
-      <c r="B41" s="37" t="s">
+      <c r="B41" s="26" t="s">
         <v>80</v>
       </c>
-      <c r="C41" s="3" t="s">
-        <v>13</v>
+      <c r="C41" s="22">
+        <v>400</v>
       </c>
       <c r="D41" s="3" t="s">
         <v>13</v>
@@ -2776,17 +2874,20 @@
       <c r="P41" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="Q41" s="23">
+      <c r="Q41" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="R41" s="22">
         <v>11</v>
       </c>
-      <c r="R41" s="23">
+      <c r="S41" s="22">
         <v>14</v>
       </c>
-      <c r="S41" s="7"/>
-    </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T41" s="7"/>
+    </row>
+    <row r="42" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A42" s="11"/>
-      <c r="B42" s="37"/>
+      <c r="B42" s="26"/>
       <c r="C42" s="3"/>
       <c r="D42" s="3"/>
       <c r="E42" s="3"/>
@@ -2803,11 +2904,12 @@
       <c r="P42" s="3"/>
       <c r="Q42" s="3"/>
       <c r="R42" s="3"/>
-      <c r="S42" s="7"/>
-    </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S42" s="3"/>
+      <c r="T42" s="7"/>
+    </row>
+    <row r="43" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A43" s="11"/>
-      <c r="B43" s="37"/>
+      <c r="B43" s="26"/>
       <c r="C43" s="3"/>
       <c r="D43" s="3"/>
       <c r="E43" s="3"/>
@@ -2824,11 +2926,12 @@
       <c r="P43" s="3"/>
       <c r="Q43" s="3"/>
       <c r="R43" s="3"/>
-      <c r="S43" s="7"/>
-    </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S43" s="3"/>
+      <c r="T43" s="7"/>
+    </row>
+    <row r="44" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A44" s="11"/>
-      <c r="B44" s="37"/>
+      <c r="B44" s="26"/>
       <c r="C44" s="3"/>
       <c r="D44" s="3"/>
       <c r="E44" s="3"/>
@@ -2845,11 +2948,12 @@
       <c r="P44" s="3"/>
       <c r="Q44" s="3"/>
       <c r="R44" s="3"/>
-      <c r="S44" s="7"/>
-    </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S44" s="3"/>
+      <c r="T44" s="7"/>
+    </row>
+    <row r="45" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A45" s="11"/>
-      <c r="B45" s="37"/>
+      <c r="B45" s="26"/>
       <c r="C45" s="3"/>
       <c r="D45" s="3"/>
       <c r="E45" s="3"/>
@@ -2866,11 +2970,12 @@
       <c r="P45" s="3"/>
       <c r="Q45" s="3"/>
       <c r="R45" s="3"/>
-      <c r="S45" s="7"/>
-    </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S45" s="3"/>
+      <c r="T45" s="7"/>
+    </row>
+    <row r="46" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A46" s="11"/>
-      <c r="B46" s="37"/>
+      <c r="B46" s="26"/>
       <c r="C46" s="3"/>
       <c r="D46" s="3"/>
       <c r="E46" s="3"/>
@@ -2887,11 +2992,12 @@
       <c r="P46" s="3"/>
       <c r="Q46" s="3"/>
       <c r="R46" s="3"/>
-      <c r="S46" s="7"/>
-    </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S46" s="3"/>
+      <c r="T46" s="7"/>
+    </row>
+    <row r="47" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A47" s="11"/>
-      <c r="B47" s="37"/>
+      <c r="B47" s="26"/>
       <c r="C47" s="3"/>
       <c r="D47" s="3"/>
       <c r="E47" s="3"/>
@@ -2908,11 +3014,12 @@
       <c r="P47" s="3"/>
       <c r="Q47" s="3"/>
       <c r="R47" s="3"/>
-      <c r="S47" s="7"/>
-    </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S47" s="3"/>
+      <c r="T47" s="7"/>
+    </row>
+    <row r="48" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A48" s="11"/>
-      <c r="B48" s="37"/>
+      <c r="B48" s="26"/>
       <c r="C48" s="3"/>
       <c r="D48" s="3"/>
       <c r="E48" s="3"/>
@@ -2929,11 +3036,12 @@
       <c r="P48" s="3"/>
       <c r="Q48" s="3"/>
       <c r="R48" s="3"/>
-      <c r="S48" s="7"/>
-    </row>
-    <row r="49" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S48" s="3"/>
+      <c r="T48" s="7"/>
+    </row>
+    <row r="49" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A49" s="11"/>
-      <c r="B49" s="37"/>
+      <c r="B49" s="26"/>
       <c r="C49" s="3"/>
       <c r="D49" s="3"/>
       <c r="E49" s="3"/>
@@ -2950,11 +3058,12 @@
       <c r="P49" s="3"/>
       <c r="Q49" s="3"/>
       <c r="R49" s="3"/>
-      <c r="S49" s="7"/>
-    </row>
-    <row r="50" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S49" s="3"/>
+      <c r="T49" s="7"/>
+    </row>
+    <row r="50" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A50" s="11"/>
-      <c r="B50" s="37"/>
+      <c r="B50" s="26"/>
       <c r="C50" s="3"/>
       <c r="D50" s="3"/>
       <c r="E50" s="3"/>
@@ -2971,11 +3080,12 @@
       <c r="P50" s="3"/>
       <c r="Q50" s="3"/>
       <c r="R50" s="3"/>
-      <c r="S50" s="7"/>
-    </row>
-    <row r="51" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S50" s="3"/>
+      <c r="T50" s="7"/>
+    </row>
+    <row r="51" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A51" s="11"/>
-      <c r="B51" s="37"/>
+      <c r="B51" s="26"/>
       <c r="C51" s="3"/>
       <c r="D51" s="3"/>
       <c r="E51" s="3"/>
@@ -2992,11 +3102,12 @@
       <c r="P51" s="3"/>
       <c r="Q51" s="3"/>
       <c r="R51" s="3"/>
-      <c r="S51" s="7"/>
-    </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S51" s="3"/>
+      <c r="T51" s="7"/>
+    </row>
+    <row r="52" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A52" s="11"/>
-      <c r="B52" s="37"/>
+      <c r="B52" s="26"/>
       <c r="C52" s="3"/>
       <c r="D52" s="3"/>
       <c r="E52" s="3"/>
@@ -3013,11 +3124,12 @@
       <c r="P52" s="3"/>
       <c r="Q52" s="3"/>
       <c r="R52" s="3"/>
-      <c r="S52" s="7"/>
-    </row>
-    <row r="53" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S52" s="3"/>
+      <c r="T52" s="7"/>
+    </row>
+    <row r="53" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A53" s="11"/>
-      <c r="B53" s="37"/>
+      <c r="B53" s="26"/>
       <c r="C53" s="3"/>
       <c r="D53" s="3"/>
       <c r="E53" s="3"/>
@@ -3034,11 +3146,12 @@
       <c r="P53" s="3"/>
       <c r="Q53" s="3"/>
       <c r="R53" s="3"/>
-      <c r="S53" s="7"/>
-    </row>
-    <row r="54" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S53" s="3"/>
+      <c r="T53" s="7"/>
+    </row>
+    <row r="54" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A54" s="11"/>
-      <c r="B54" s="37"/>
+      <c r="B54" s="26"/>
       <c r="C54" s="3"/>
       <c r="D54" s="3"/>
       <c r="E54" s="3"/>
@@ -3055,11 +3168,12 @@
       <c r="P54" s="3"/>
       <c r="Q54" s="3"/>
       <c r="R54" s="3"/>
-      <c r="S54" s="7"/>
-    </row>
-    <row r="55" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S54" s="3"/>
+      <c r="T54" s="7"/>
+    </row>
+    <row r="55" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A55" s="11"/>
-      <c r="B55" s="37"/>
+      <c r="B55" s="26"/>
       <c r="C55" s="3"/>
       <c r="D55" s="3"/>
       <c r="E55" s="3"/>
@@ -3076,11 +3190,12 @@
       <c r="P55" s="3"/>
       <c r="Q55" s="3"/>
       <c r="R55" s="3"/>
-      <c r="S55" s="7"/>
-    </row>
-    <row r="56" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S55" s="3"/>
+      <c r="T55" s="7"/>
+    </row>
+    <row r="56" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A56" s="11"/>
-      <c r="B56" s="37"/>
+      <c r="B56" s="26"/>
       <c r="C56" s="3"/>
       <c r="D56" s="3"/>
       <c r="E56" s="3"/>
@@ -3097,11 +3212,12 @@
       <c r="P56" s="3"/>
       <c r="Q56" s="3"/>
       <c r="R56" s="3"/>
-      <c r="S56" s="7"/>
-    </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S56" s="3"/>
+      <c r="T56" s="7"/>
+    </row>
+    <row r="57" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A57" s="11"/>
-      <c r="B57" s="37"/>
+      <c r="B57" s="26"/>
       <c r="C57" s="3"/>
       <c r="D57" s="3"/>
       <c r="E57" s="3"/>
@@ -3118,11 +3234,12 @@
       <c r="P57" s="3"/>
       <c r="Q57" s="3"/>
       <c r="R57" s="3"/>
-      <c r="S57" s="7"/>
-    </row>
-    <row r="58" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S57" s="3"/>
+      <c r="T57" s="7"/>
+    </row>
+    <row r="58" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A58" s="11"/>
-      <c r="B58" s="37"/>
+      <c r="B58" s="26"/>
       <c r="C58" s="3"/>
       <c r="D58" s="3"/>
       <c r="E58" s="3"/>
@@ -3139,11 +3256,12 @@
       <c r="P58" s="3"/>
       <c r="Q58" s="3"/>
       <c r="R58" s="3"/>
-      <c r="S58" s="7"/>
-    </row>
-    <row r="59" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S58" s="3"/>
+      <c r="T58" s="7"/>
+    </row>
+    <row r="59" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A59" s="11"/>
-      <c r="B59" s="37"/>
+      <c r="B59" s="26"/>
       <c r="C59" s="3"/>
       <c r="D59" s="3"/>
       <c r="E59" s="3"/>
@@ -3160,11 +3278,12 @@
       <c r="P59" s="3"/>
       <c r="Q59" s="3"/>
       <c r="R59" s="3"/>
-      <c r="S59" s="7"/>
-    </row>
-    <row r="60" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S59" s="3"/>
+      <c r="T59" s="7"/>
+    </row>
+    <row r="60" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A60" s="11"/>
-      <c r="B60" s="37"/>
+      <c r="B60" s="26"/>
       <c r="C60" s="3"/>
       <c r="D60" s="3"/>
       <c r="E60" s="3"/>
@@ -3181,11 +3300,12 @@
       <c r="P60" s="3"/>
       <c r="Q60" s="3"/>
       <c r="R60" s="3"/>
-      <c r="S60" s="7"/>
-    </row>
-    <row r="61" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S60" s="3"/>
+      <c r="T60" s="7"/>
+    </row>
+    <row r="61" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A61" s="11"/>
-      <c r="B61" s="37"/>
+      <c r="B61" s="26"/>
       <c r="C61" s="3"/>
       <c r="D61" s="3"/>
       <c r="E61" s="3"/>
@@ -3202,11 +3322,12 @@
       <c r="P61" s="3"/>
       <c r="Q61" s="3"/>
       <c r="R61" s="3"/>
-      <c r="S61" s="7"/>
-    </row>
-    <row r="62" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S61" s="3"/>
+      <c r="T61" s="7"/>
+    </row>
+    <row r="62" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A62" s="11"/>
-      <c r="B62" s="37"/>
+      <c r="B62" s="26"/>
       <c r="C62" s="3"/>
       <c r="D62" s="3"/>
       <c r="E62" s="3"/>
@@ -3223,11 +3344,12 @@
       <c r="P62" s="3"/>
       <c r="Q62" s="3"/>
       <c r="R62" s="3"/>
-      <c r="S62" s="7"/>
-    </row>
-    <row r="63" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S62" s="3"/>
+      <c r="T62" s="7"/>
+    </row>
+    <row r="63" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A63" s="11"/>
-      <c r="B63" s="37"/>
+      <c r="B63" s="26"/>
       <c r="C63" s="3"/>
       <c r="D63" s="3"/>
       <c r="E63" s="3"/>
@@ -3244,11 +3366,12 @@
       <c r="P63" s="3"/>
       <c r="Q63" s="3"/>
       <c r="R63" s="3"/>
-      <c r="S63" s="7"/>
-    </row>
-    <row r="64" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S63" s="3"/>
+      <c r="T63" s="7"/>
+    </row>
+    <row r="64" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A64" s="11"/>
-      <c r="B64" s="37"/>
+      <c r="B64" s="26"/>
       <c r="C64" s="3"/>
       <c r="D64" s="3"/>
       <c r="E64" s="3"/>
@@ -3265,11 +3388,12 @@
       <c r="P64" s="3"/>
       <c r="Q64" s="3"/>
       <c r="R64" s="3"/>
-      <c r="S64" s="7"/>
-    </row>
-    <row r="65" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S64" s="3"/>
+      <c r="T64" s="7"/>
+    </row>
+    <row r="65" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A65" s="11"/>
-      <c r="B65" s="37"/>
+      <c r="B65" s="26"/>
       <c r="C65" s="3"/>
       <c r="D65" s="3"/>
       <c r="E65" s="3"/>
@@ -3286,11 +3410,12 @@
       <c r="P65" s="3"/>
       <c r="Q65" s="3"/>
       <c r="R65" s="3"/>
-      <c r="S65" s="7"/>
-    </row>
-    <row r="66" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S65" s="3"/>
+      <c r="T65" s="7"/>
+    </row>
+    <row r="66" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A66" s="11"/>
-      <c r="B66" s="37"/>
+      <c r="B66" s="26"/>
       <c r="C66" s="3"/>
       <c r="D66" s="3"/>
       <c r="E66" s="3"/>
@@ -3307,11 +3432,12 @@
       <c r="P66" s="3"/>
       <c r="Q66" s="3"/>
       <c r="R66" s="3"/>
-      <c r="S66" s="7"/>
-    </row>
-    <row r="67" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S66" s="3"/>
+      <c r="T66" s="7"/>
+    </row>
+    <row r="67" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A67" s="11"/>
-      <c r="B67" s="37"/>
+      <c r="B67" s="26"/>
       <c r="C67" s="3"/>
       <c r="D67" s="3"/>
       <c r="E67" s="3"/>
@@ -3328,11 +3454,12 @@
       <c r="P67" s="3"/>
       <c r="Q67" s="3"/>
       <c r="R67" s="3"/>
-      <c r="S67" s="7"/>
-    </row>
-    <row r="68" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S67" s="3"/>
+      <c r="T67" s="7"/>
+    </row>
+    <row r="68" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A68" s="11"/>
-      <c r="B68" s="37"/>
+      <c r="B68" s="26"/>
       <c r="C68" s="3"/>
       <c r="D68" s="3"/>
       <c r="E68" s="3"/>
@@ -3349,11 +3476,12 @@
       <c r="P68" s="3"/>
       <c r="Q68" s="3"/>
       <c r="R68" s="3"/>
-      <c r="S68" s="7"/>
-    </row>
-    <row r="69" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S68" s="3"/>
+      <c r="T68" s="7"/>
+    </row>
+    <row r="69" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A69" s="11"/>
-      <c r="B69" s="37"/>
+      <c r="B69" s="26"/>
       <c r="C69" s="3"/>
       <c r="D69" s="3"/>
       <c r="E69" s="3"/>
@@ -3370,11 +3498,12 @@
       <c r="P69" s="3"/>
       <c r="Q69" s="3"/>
       <c r="R69" s="3"/>
-      <c r="S69" s="7"/>
-    </row>
-    <row r="70" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S69" s="3"/>
+      <c r="T69" s="7"/>
+    </row>
+    <row r="70" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A70" s="11"/>
-      <c r="B70" s="37"/>
+      <c r="B70" s="26"/>
       <c r="C70" s="3"/>
       <c r="D70" s="3"/>
       <c r="E70" s="3"/>
@@ -3391,11 +3520,12 @@
       <c r="P70" s="3"/>
       <c r="Q70" s="3"/>
       <c r="R70" s="3"/>
-      <c r="S70" s="7"/>
-    </row>
-    <row r="71" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S70" s="3"/>
+      <c r="T70" s="7"/>
+    </row>
+    <row r="71" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A71" s="11"/>
-      <c r="B71" s="37"/>
+      <c r="B71" s="26"/>
       <c r="C71" s="3"/>
       <c r="D71" s="3"/>
       <c r="E71" s="3"/>
@@ -3412,11 +3542,12 @@
       <c r="P71" s="3"/>
       <c r="Q71" s="3"/>
       <c r="R71" s="3"/>
-      <c r="S71" s="7"/>
-    </row>
-    <row r="72" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S71" s="3"/>
+      <c r="T71" s="7"/>
+    </row>
+    <row r="72" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A72" s="11"/>
-      <c r="B72" s="37"/>
+      <c r="B72" s="26"/>
       <c r="C72" s="3"/>
       <c r="D72" s="3"/>
       <c r="E72" s="3"/>
@@ -3433,11 +3564,12 @@
       <c r="P72" s="3"/>
       <c r="Q72" s="3"/>
       <c r="R72" s="3"/>
-      <c r="S72" s="7"/>
-    </row>
-    <row r="73" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S72" s="3"/>
+      <c r="T72" s="7"/>
+    </row>
+    <row r="73" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A73" s="11"/>
-      <c r="B73" s="37"/>
+      <c r="B73" s="26"/>
       <c r="C73" s="3"/>
       <c r="D73" s="3"/>
       <c r="E73" s="3"/>
@@ -3454,11 +3586,12 @@
       <c r="P73" s="3"/>
       <c r="Q73" s="3"/>
       <c r="R73" s="3"/>
-      <c r="S73" s="7"/>
-    </row>
-    <row r="74" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S73" s="3"/>
+      <c r="T73" s="7"/>
+    </row>
+    <row r="74" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A74" s="11"/>
-      <c r="B74" s="37"/>
+      <c r="B74" s="26"/>
       <c r="C74" s="3"/>
       <c r="D74" s="3"/>
       <c r="E74" s="3"/>
@@ -3475,11 +3608,12 @@
       <c r="P74" s="3"/>
       <c r="Q74" s="3"/>
       <c r="R74" s="3"/>
-      <c r="S74" s="7"/>
-    </row>
-    <row r="75" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S74" s="3"/>
+      <c r="T74" s="7"/>
+    </row>
+    <row r="75" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A75" s="11"/>
-      <c r="B75" s="37"/>
+      <c r="B75" s="26"/>
       <c r="C75" s="3"/>
       <c r="D75" s="3"/>
       <c r="E75" s="3"/>
@@ -3496,11 +3630,12 @@
       <c r="P75" s="3"/>
       <c r="Q75" s="3"/>
       <c r="R75" s="3"/>
-      <c r="S75" s="7"/>
-    </row>
-    <row r="76" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S75" s="3"/>
+      <c r="T75" s="7"/>
+    </row>
+    <row r="76" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A76" s="11"/>
-      <c r="B76" s="37"/>
+      <c r="B76" s="26"/>
       <c r="C76" s="3"/>
       <c r="D76" s="3"/>
       <c r="E76" s="3"/>
@@ -3517,11 +3652,12 @@
       <c r="P76" s="3"/>
       <c r="Q76" s="3"/>
       <c r="R76" s="3"/>
-      <c r="S76" s="7"/>
-    </row>
-    <row r="77" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S76" s="3"/>
+      <c r="T76" s="7"/>
+    </row>
+    <row r="77" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A77" s="11"/>
-      <c r="B77" s="37"/>
+      <c r="B77" s="26"/>
       <c r="C77" s="3"/>
       <c r="D77" s="3"/>
       <c r="E77" s="3"/>
@@ -3538,11 +3674,12 @@
       <c r="P77" s="3"/>
       <c r="Q77" s="3"/>
       <c r="R77" s="3"/>
-      <c r="S77" s="7"/>
-    </row>
-    <row r="78" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S77" s="3"/>
+      <c r="T77" s="7"/>
+    </row>
+    <row r="78" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A78" s="11"/>
-      <c r="B78" s="37"/>
+      <c r="B78" s="26"/>
       <c r="C78" s="3"/>
       <c r="D78" s="3"/>
       <c r="E78" s="3"/>
@@ -3559,11 +3696,12 @@
       <c r="P78" s="3"/>
       <c r="Q78" s="3"/>
       <c r="R78" s="3"/>
-      <c r="S78" s="7"/>
-    </row>
-    <row r="79" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S78" s="3"/>
+      <c r="T78" s="7"/>
+    </row>
+    <row r="79" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A79" s="11"/>
-      <c r="B79" s="37"/>
+      <c r="B79" s="26"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
       <c r="E79" s="3"/>
@@ -3580,11 +3718,12 @@
       <c r="P79" s="3"/>
       <c r="Q79" s="3"/>
       <c r="R79" s="3"/>
-      <c r="S79" s="7"/>
-    </row>
-    <row r="80" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S79" s="3"/>
+      <c r="T79" s="7"/>
+    </row>
+    <row r="80" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A80" s="11"/>
-      <c r="B80" s="37"/>
+      <c r="B80" s="26"/>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
       <c r="E80" s="3"/>
@@ -3601,11 +3740,12 @@
       <c r="P80" s="3"/>
       <c r="Q80" s="3"/>
       <c r="R80" s="3"/>
-      <c r="S80" s="7"/>
-    </row>
-    <row r="81" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S80" s="3"/>
+      <c r="T80" s="7"/>
+    </row>
+    <row r="81" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A81" s="11"/>
-      <c r="B81" s="37"/>
+      <c r="B81" s="26"/>
       <c r="C81" s="3"/>
       <c r="D81" s="3"/>
       <c r="E81" s="3"/>
@@ -3622,11 +3762,12 @@
       <c r="P81" s="3"/>
       <c r="Q81" s="3"/>
       <c r="R81" s="3"/>
-      <c r="S81" s="7"/>
-    </row>
-    <row r="82" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S81" s="3"/>
+      <c r="T81" s="7"/>
+    </row>
+    <row r="82" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A82" s="11"/>
-      <c r="B82" s="37"/>
+      <c r="B82" s="26"/>
       <c r="C82" s="3"/>
       <c r="D82" s="3"/>
       <c r="E82" s="3"/>
@@ -3643,11 +3784,12 @@
       <c r="P82" s="3"/>
       <c r="Q82" s="3"/>
       <c r="R82" s="3"/>
-      <c r="S82" s="7"/>
-    </row>
-    <row r="83" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S82" s="3"/>
+      <c r="T82" s="7"/>
+    </row>
+    <row r="83" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A83" s="11"/>
-      <c r="B83" s="37"/>
+      <c r="B83" s="26"/>
       <c r="C83" s="3"/>
       <c r="D83" s="3"/>
       <c r="E83" s="3"/>
@@ -3664,11 +3806,12 @@
       <c r="P83" s="3"/>
       <c r="Q83" s="3"/>
       <c r="R83" s="3"/>
-      <c r="S83" s="7"/>
-    </row>
-    <row r="84" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S83" s="3"/>
+      <c r="T83" s="7"/>
+    </row>
+    <row r="84" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A84" s="11"/>
-      <c r="B84" s="37"/>
+      <c r="B84" s="26"/>
       <c r="C84" s="3"/>
       <c r="D84" s="3"/>
       <c r="E84" s="3"/>
@@ -3685,11 +3828,12 @@
       <c r="P84" s="3"/>
       <c r="Q84" s="3"/>
       <c r="R84" s="3"/>
-      <c r="S84" s="7"/>
-    </row>
-    <row r="85" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S84" s="3"/>
+      <c r="T84" s="7"/>
+    </row>
+    <row r="85" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A85" s="11"/>
-      <c r="B85" s="37"/>
+      <c r="B85" s="26"/>
       <c r="C85" s="3"/>
       <c r="D85" s="3"/>
       <c r="E85" s="3"/>
@@ -3706,11 +3850,12 @@
       <c r="P85" s="3"/>
       <c r="Q85" s="3"/>
       <c r="R85" s="3"/>
-      <c r="S85" s="7"/>
-    </row>
-    <row r="86" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S85" s="3"/>
+      <c r="T85" s="7"/>
+    </row>
+    <row r="86" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A86" s="11"/>
-      <c r="B86" s="37"/>
+      <c r="B86" s="26"/>
       <c r="C86" s="3"/>
       <c r="D86" s="3"/>
       <c r="E86" s="3"/>
@@ -3727,11 +3872,12 @@
       <c r="P86" s="3"/>
       <c r="Q86" s="3"/>
       <c r="R86" s="3"/>
-      <c r="S86" s="7"/>
-    </row>
-    <row r="87" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S86" s="3"/>
+      <c r="T86" s="7"/>
+    </row>
+    <row r="87" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A87" s="11"/>
-      <c r="B87" s="37"/>
+      <c r="B87" s="26"/>
       <c r="C87" s="3"/>
       <c r="D87" s="3"/>
       <c r="E87" s="3"/>
@@ -3748,11 +3894,12 @@
       <c r="P87" s="3"/>
       <c r="Q87" s="3"/>
       <c r="R87" s="3"/>
-      <c r="S87" s="7"/>
-    </row>
-    <row r="88" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S87" s="3"/>
+      <c r="T87" s="7"/>
+    </row>
+    <row r="88" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A88" s="11"/>
-      <c r="B88" s="37"/>
+      <c r="B88" s="26"/>
       <c r="C88" s="3"/>
       <c r="D88" s="3"/>
       <c r="E88" s="3"/>
@@ -3769,11 +3916,12 @@
       <c r="P88" s="3"/>
       <c r="Q88" s="3"/>
       <c r="R88" s="3"/>
-      <c r="S88" s="7"/>
-    </row>
-    <row r="89" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S88" s="3"/>
+      <c r="T88" s="7"/>
+    </row>
+    <row r="89" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A89" s="11"/>
-      <c r="B89" s="37"/>
+      <c r="B89" s="26"/>
       <c r="C89" s="3"/>
       <c r="D89" s="3"/>
       <c r="E89" s="3"/>
@@ -3790,11 +3938,12 @@
       <c r="P89" s="3"/>
       <c r="Q89" s="3"/>
       <c r="R89" s="3"/>
-      <c r="S89" s="7"/>
-    </row>
-    <row r="90" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S89" s="3"/>
+      <c r="T89" s="7"/>
+    </row>
+    <row r="90" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A90" s="11"/>
-      <c r="B90" s="37"/>
+      <c r="B90" s="26"/>
       <c r="C90" s="3"/>
       <c r="D90" s="3"/>
       <c r="E90" s="3"/>
@@ -3811,11 +3960,12 @@
       <c r="P90" s="3"/>
       <c r="Q90" s="3"/>
       <c r="R90" s="3"/>
-      <c r="S90" s="7"/>
-    </row>
-    <row r="91" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S90" s="3"/>
+      <c r="T90" s="7"/>
+    </row>
+    <row r="91" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A91" s="11"/>
-      <c r="B91" s="37"/>
+      <c r="B91" s="26"/>
       <c r="C91" s="3"/>
       <c r="D91" s="3"/>
       <c r="E91" s="3"/>
@@ -3832,11 +3982,12 @@
       <c r="P91" s="3"/>
       <c r="Q91" s="3"/>
       <c r="R91" s="3"/>
-      <c r="S91" s="7"/>
-    </row>
-    <row r="92" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S91" s="3"/>
+      <c r="T91" s="7"/>
+    </row>
+    <row r="92" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A92" s="11"/>
-      <c r="B92" s="37"/>
+      <c r="B92" s="26"/>
       <c r="C92" s="3"/>
       <c r="D92" s="3"/>
       <c r="E92" s="3"/>
@@ -3853,11 +4004,12 @@
       <c r="P92" s="3"/>
       <c r="Q92" s="3"/>
       <c r="R92" s="3"/>
-      <c r="S92" s="7"/>
-    </row>
-    <row r="93" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S92" s="3"/>
+      <c r="T92" s="7"/>
+    </row>
+    <row r="93" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A93" s="11"/>
-      <c r="B93" s="37"/>
+      <c r="B93" s="26"/>
       <c r="C93" s="3"/>
       <c r="D93" s="3"/>
       <c r="E93" s="3"/>
@@ -3874,11 +4026,12 @@
       <c r="P93" s="3"/>
       <c r="Q93" s="3"/>
       <c r="R93" s="3"/>
-      <c r="S93" s="7"/>
-    </row>
-    <row r="94" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S93" s="3"/>
+      <c r="T93" s="7"/>
+    </row>
+    <row r="94" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A94" s="11"/>
-      <c r="B94" s="37"/>
+      <c r="B94" s="26"/>
       <c r="C94" s="3"/>
       <c r="D94" s="3"/>
       <c r="E94" s="3"/>
@@ -3895,11 +4048,12 @@
       <c r="P94" s="3"/>
       <c r="Q94" s="3"/>
       <c r="R94" s="3"/>
-      <c r="S94" s="7"/>
-    </row>
-    <row r="95" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S94" s="3"/>
+      <c r="T94" s="7"/>
+    </row>
+    <row r="95" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A95" s="11"/>
-      <c r="B95" s="37"/>
+      <c r="B95" s="26"/>
       <c r="C95" s="3"/>
       <c r="D95" s="3"/>
       <c r="E95" s="3"/>
@@ -3916,11 +4070,12 @@
       <c r="P95" s="3"/>
       <c r="Q95" s="3"/>
       <c r="R95" s="3"/>
-      <c r="S95" s="7"/>
-    </row>
-    <row r="96" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S95" s="3"/>
+      <c r="T95" s="7"/>
+    </row>
+    <row r="96" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A96" s="11"/>
-      <c r="B96" s="37"/>
+      <c r="B96" s="26"/>
       <c r="C96" s="3"/>
       <c r="D96" s="3"/>
       <c r="E96" s="3"/>
@@ -3937,11 +4092,12 @@
       <c r="P96" s="3"/>
       <c r="Q96" s="3"/>
       <c r="R96" s="3"/>
-      <c r="S96" s="7"/>
-    </row>
-    <row r="97" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S96" s="3"/>
+      <c r="T96" s="7"/>
+    </row>
+    <row r="97" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A97" s="11"/>
-      <c r="B97" s="37"/>
+      <c r="B97" s="26"/>
       <c r="C97" s="3"/>
       <c r="D97" s="3"/>
       <c r="E97" s="3"/>
@@ -3958,11 +4114,12 @@
       <c r="P97" s="3"/>
       <c r="Q97" s="3"/>
       <c r="R97" s="3"/>
-      <c r="S97" s="7"/>
-    </row>
-    <row r="98" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S97" s="3"/>
+      <c r="T97" s="7"/>
+    </row>
+    <row r="98" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A98" s="11"/>
-      <c r="B98" s="37"/>
+      <c r="B98" s="26"/>
       <c r="C98" s="3"/>
       <c r="D98" s="3"/>
       <c r="E98" s="3"/>
@@ -3979,11 +4136,12 @@
       <c r="P98" s="3"/>
       <c r="Q98" s="3"/>
       <c r="R98" s="3"/>
-      <c r="S98" s="7"/>
-    </row>
-    <row r="99" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S98" s="3"/>
+      <c r="T98" s="7"/>
+    </row>
+    <row r="99" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A99" s="11"/>
-      <c r="B99" s="37"/>
+      <c r="B99" s="26"/>
       <c r="C99" s="3"/>
       <c r="D99" s="3"/>
       <c r="E99" s="3"/>
@@ -4000,11 +4158,12 @@
       <c r="P99" s="3"/>
       <c r="Q99" s="3"/>
       <c r="R99" s="3"/>
-      <c r="S99" s="7"/>
-    </row>
-    <row r="100" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S99" s="3"/>
+      <c r="T99" s="7"/>
+    </row>
+    <row r="100" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A100" s="12"/>
-      <c r="B100" s="43"/>
+      <c r="B100" s="29"/>
       <c r="C100" s="8"/>
       <c r="D100" s="8"/>
       <c r="E100" s="8"/>
@@ -4021,27 +4180,28 @@
       <c r="P100" s="8"/>
       <c r="Q100" s="8"/>
       <c r="R100" s="8"/>
-      <c r="S100" s="9"/>
+      <c r="S100" s="8"/>
+      <c r="T100" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="D1:G1"/>
+    <mergeCell ref="D2:G2"/>
+    <mergeCell ref="D5:G5"/>
+    <mergeCell ref="D4:G4"/>
+    <mergeCell ref="D3:G3"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A8:A10"/>
     <mergeCell ref="B8:B10"/>
-    <mergeCell ref="S8:S9"/>
-    <mergeCell ref="C1:F1"/>
-    <mergeCell ref="C2:F2"/>
-    <mergeCell ref="C5:F5"/>
-    <mergeCell ref="C4:F4"/>
-    <mergeCell ref="C3:F3"/>
-    <mergeCell ref="P8:R8"/>
-    <mergeCell ref="C8:F8"/>
-    <mergeCell ref="G8:O8"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="T8:T9"/>
+    <mergeCell ref="Q8:S8"/>
+    <mergeCell ref="H8:P8"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>